<commit_message>
ingesta: snapshot 2026-10-25 18:19 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-10-25/Temp-max-octubre-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-10-25/Temp-max-octubre-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7785733A-7765-4954-974B-696541DC7E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C067A03-F98C-47CC-8163-DC8FE0BA5E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TMAX_PRINCIPALES_CIUDADES" sheetId="1" r:id="rId1"/>
@@ -1070,7 +1070,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1122,6 +1122,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1210,7 +1216,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1435,6 +1441,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -9495,7 +9504,9 @@
       <c r="AA5" s="63">
         <v>31</v>
       </c>
-      <c r="AB5" s="63"/>
+      <c r="AB5" s="63">
+        <v>30.7</v>
+      </c>
       <c r="AC5" s="63"/>
       <c r="AD5" s="63"/>
       <c r="AE5" s="63"/>
@@ -9505,7 +9516,7 @@
       <c r="AI5" s="63"/>
       <c r="AJ5" s="36">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>31</v>
+        <v>30.7</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9523,11 +9534,11 @@
       </c>
       <c r="AO5" s="23">
         <f>IF(COUNTIF(E5:AI5,"&gt;0")&gt;=15,AVERAGE(E5:AI5),"")</f>
-        <v>31.795652173913041</v>
+        <v>31.75</v>
       </c>
       <c r="AP5" s="23">
         <f>IF(AN5&gt;0,IFERROR(AO5-AN5,""),"")</f>
-        <v>1.3522927432065615</v>
+        <v>1.3066405692935206</v>
       </c>
       <c r="AQ5" s="20"/>
     </row>
@@ -9613,7 +9624,9 @@
       <c r="AA6" s="63">
         <v>29.1</v>
       </c>
-      <c r="AB6" s="63"/>
+      <c r="AB6" s="63">
+        <v>31.1</v>
+      </c>
       <c r="AC6" s="63"/>
       <c r="AD6" s="63"/>
       <c r="AE6" s="63"/>
@@ -9623,7 +9636,7 @@
       <c r="AI6" s="63"/>
       <c r="AJ6" s="36">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>29.1</v>
+        <v>31.1</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
@@ -9641,11 +9654,11 @@
       </c>
       <c r="AO6" s="23">
         <f t="shared" ref="AO6:AO15" si="3">IF(COUNTIF(E6:AI6,"&gt;0")&gt;=15,AVERAGE(E6:AI6),"")</f>
-        <v>31.460869565217394</v>
+        <v>31.445833333333336</v>
       </c>
       <c r="AP6" s="23">
         <f t="shared" ref="AP6:AP48" si="4">IF(AN6&gt;0,IFERROR(AO6-AN6,""),"")</f>
-        <v>0.74302102188497443</v>
+        <v>0.72798479000091731</v>
       </c>
       <c r="AQ6" s="20"/>
     </row>
@@ -9731,7 +9744,9 @@
       <c r="AA7" s="63">
         <v>34.6</v>
       </c>
-      <c r="AB7" s="63"/>
+      <c r="AB7" s="63">
+        <v>34</v>
+      </c>
       <c r="AC7" s="63"/>
       <c r="AD7" s="63"/>
       <c r="AE7" s="63"/>
@@ -9741,7 +9756,7 @@
       <c r="AI7" s="63"/>
       <c r="AJ7" s="36">
         <f t="shared" si="0"/>
-        <v>34.6</v>
+        <v>34</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9759,11 +9774,11 @@
       </c>
       <c r="AO7" s="23">
         <f t="shared" si="3"/>
-        <v>33.844782608695652</v>
+        <v>33.85125</v>
       </c>
       <c r="AP7" s="23">
         <f t="shared" si="4"/>
-        <v>1.4031712220201058</v>
+        <v>1.4096386133244536</v>
       </c>
       <c r="AQ7" s="20"/>
     </row>
@@ -9849,7 +9864,9 @@
       <c r="AA8" s="63">
         <v>33.299999999999997</v>
       </c>
-      <c r="AB8" s="63"/>
+      <c r="AB8" s="63">
+        <v>30.8</v>
+      </c>
       <c r="AC8" s="63"/>
       <c r="AD8" s="63"/>
       <c r="AE8" s="63"/>
@@ -9859,7 +9876,7 @@
       <c r="AI8" s="63"/>
       <c r="AJ8" s="36">
         <f t="shared" si="0"/>
-        <v>33.299999999999997</v>
+        <v>30.8</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9877,11 +9894,11 @@
       </c>
       <c r="AO8" s="23">
         <f t="shared" si="3"/>
-        <v>32.578260869565227</v>
+        <v>32.50416666666667</v>
       </c>
       <c r="AP8" s="23">
         <f t="shared" si="4"/>
-        <v>0.90868356144509832</v>
+        <v>0.83458935854654115</v>
       </c>
       <c r="AQ8" s="20"/>
     </row>
@@ -9967,7 +9984,9 @@
       <c r="AA9" s="63">
         <v>35.799999999999997</v>
       </c>
-      <c r="AB9" s="63"/>
+      <c r="AB9" s="63">
+        <v>32.200000000000003</v>
+      </c>
       <c r="AC9" s="63"/>
       <c r="AD9" s="63"/>
       <c r="AE9" s="63"/>
@@ -9977,7 +9996,7 @@
       <c r="AI9" s="63"/>
       <c r="AJ9" s="36">
         <f t="shared" si="0"/>
-        <v>35.799999999999997</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9995,11 +10014,11 @@
       </c>
       <c r="AO9" s="23">
         <f t="shared" si="3"/>
-        <v>34.199999999999996</v>
+        <v>34.116666666666667</v>
       </c>
       <c r="AP9" s="23">
         <f t="shared" si="4"/>
-        <v>1.4382361425648682</v>
+        <v>1.3549028092315396</v>
       </c>
       <c r="AQ9" s="20"/>
     </row>
@@ -10085,7 +10104,9 @@
       <c r="AA10" s="63">
         <v>33.799999999999997</v>
       </c>
-      <c r="AB10" s="63"/>
+      <c r="AB10" s="63">
+        <v>32.299999999999997</v>
+      </c>
       <c r="AC10" s="63"/>
       <c r="AD10" s="63"/>
       <c r="AE10" s="63"/>
@@ -10095,7 +10116,7 @@
       <c r="AI10" s="63"/>
       <c r="AJ10" s="36">
         <f t="shared" si="0"/>
-        <v>33.799999999999997</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -10113,11 +10134,11 @@
       </c>
       <c r="AO10" s="23">
         <f t="shared" si="3"/>
-        <v>33.804347826086953</v>
+        <v>33.74166666666666</v>
       </c>
       <c r="AP10" s="23">
         <f t="shared" si="4"/>
-        <v>1.0183834703780406</v>
+        <v>0.95570231095774716</v>
       </c>
       <c r="AQ10" s="20"/>
     </row>
@@ -10203,7 +10224,9 @@
       <c r="AA11" s="63">
         <v>35.4</v>
       </c>
-      <c r="AB11" s="63"/>
+      <c r="AB11" s="63">
+        <v>33.299999999999997</v>
+      </c>
       <c r="AC11" s="63"/>
       <c r="AD11" s="63"/>
       <c r="AE11" s="63"/>
@@ -10213,7 +10236,7 @@
       <c r="AI11" s="63"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
-        <v>35.4</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -10231,11 +10254,11 @@
       </c>
       <c r="AO11" s="23">
         <f t="shared" si="3"/>
-        <v>34.486956521739124</v>
+        <v>34.437499999999993</v>
       </c>
       <c r="AP11" s="23">
         <f t="shared" si="4"/>
-        <v>1.4495092895607016</v>
+        <v>1.4000527678215704</v>
       </c>
       <c r="AQ11" s="20"/>
     </row>
@@ -10321,7 +10344,9 @@
       <c r="AA12" s="63">
         <v>33.6</v>
       </c>
-      <c r="AB12" s="63"/>
+      <c r="AB12" s="83">
+        <v>26.6</v>
+      </c>
       <c r="AC12" s="63"/>
       <c r="AD12" s="63"/>
       <c r="AE12" s="63"/>
@@ -10331,7 +10356,7 @@
       <c r="AI12" s="63"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
-        <v>33.6</v>
+        <v>26.6</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10349,11 +10374,11 @@
       </c>
       <c r="AO12" s="23">
         <f t="shared" si="3"/>
-        <v>31.582608695652176</v>
+        <v>31.375000000000004</v>
       </c>
       <c r="AP12" s="23">
         <f t="shared" si="4"/>
-        <v>0.4703147888421455</v>
+        <v>0.26270609318997273</v>
       </c>
       <c r="AQ12" s="20"/>
     </row>
@@ -10439,7 +10464,9 @@
       <c r="AA13" s="63">
         <v>34.200000000000003</v>
       </c>
-      <c r="AB13" s="63"/>
+      <c r="AB13" s="83">
+        <v>26.6</v>
+      </c>
       <c r="AC13" s="63"/>
       <c r="AD13" s="63"/>
       <c r="AE13" s="63"/>
@@ -10449,7 +10476,7 @@
       <c r="AI13" s="63"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
-        <v>34.200000000000003</v>
+        <v>26.6</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10467,11 +10494,11 @@
       </c>
       <c r="AO13" s="23">
         <f t="shared" si="3"/>
-        <v>32.417391304347824</v>
+        <v>32.175000000000004</v>
       </c>
       <c r="AP13" s="23">
         <f t="shared" si="4"/>
-        <v>0.73305797101449244</v>
+        <v>0.49066666666667302</v>
       </c>
       <c r="AQ13" s="20"/>
     </row>
@@ -10557,7 +10584,9 @@
       <c r="AA14" s="63">
         <v>33.9</v>
       </c>
-      <c r="AB14" s="63"/>
+      <c r="AB14" s="63">
+        <v>25.5</v>
+      </c>
       <c r="AC14" s="63"/>
       <c r="AD14" s="63"/>
       <c r="AE14" s="63"/>
@@ -10567,7 +10596,7 @@
       <c r="AI14" s="63"/>
       <c r="AJ14" s="36">
         <f t="shared" si="0"/>
-        <v>33.9</v>
+        <v>25.5</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10585,11 +10614,11 @@
       </c>
       <c r="AO14" s="23">
         <f t="shared" si="3"/>
-        <v>32.678260869565221</v>
+        <v>32.37916666666667</v>
       </c>
       <c r="AP14" s="23">
         <f t="shared" si="4"/>
-        <v>0.235035038491894</v>
+        <v>-6.4059164406657487E-2</v>
       </c>
       <c r="AQ14" s="20"/>
     </row>
@@ -10675,7 +10704,9 @@
       <c r="AA15" s="63">
         <v>31.5</v>
       </c>
-      <c r="AB15" s="63"/>
+      <c r="AB15" s="63">
+        <v>29.4</v>
+      </c>
       <c r="AC15" s="63"/>
       <c r="AD15" s="63"/>
       <c r="AE15" s="63"/>
@@ -10685,7 +10716,7 @@
       <c r="AI15" s="63"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
-        <v>31.5</v>
+        <v>29.4</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10703,11 +10734,11 @@
       </c>
       <c r="AO15" s="23">
         <f t="shared" si="3"/>
-        <v>31.691304347826087</v>
+        <v>31.595833333333331</v>
       </c>
       <c r="AP15" s="23">
         <f t="shared" si="4"/>
-        <v>-5.3694693254044523E-2</v>
+        <v>-0.14916570774679982</v>
       </c>
       <c r="AQ15" s="20"/>
     </row>
@@ -10842,7 +10873,9 @@
       <c r="AA17" s="63">
         <v>35.4</v>
       </c>
-      <c r="AB17" s="63"/>
+      <c r="AB17" s="63">
+        <v>29.2</v>
+      </c>
       <c r="AC17" s="63"/>
       <c r="AD17" s="63"/>
       <c r="AE17" s="63"/>
@@ -10852,7 +10885,7 @@
       <c r="AI17" s="63"/>
       <c r="AJ17" s="36">
         <f t="shared" si="0"/>
-        <v>35.4</v>
+        <v>29.2</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10870,11 +10903,11 @@
       </c>
       <c r="AO17" s="23">
         <f>IF(COUNTIF(E17:AI17,"&gt;0")&gt;=15,AVERAGE(E17:AI17),"")</f>
-        <v>32.043478260869563</v>
+        <v>31.925000000000001</v>
       </c>
       <c r="AP17" s="23">
         <f>IF(AN17&gt;0,IFERROR(AO17-AN17,""),"")</f>
-        <v>0.60914810945415354</v>
+        <v>0.49066984858459151</v>
       </c>
       <c r="AQ17" s="20"/>
     </row>
@@ -10960,7 +10993,9 @@
       <c r="AA18" s="63">
         <v>30.2</v>
       </c>
-      <c r="AB18" s="63"/>
+      <c r="AB18" s="63">
+        <v>27.4</v>
+      </c>
       <c r="AC18" s="63"/>
       <c r="AD18" s="63"/>
       <c r="AE18" s="63"/>
@@ -10970,7 +11005,7 @@
       <c r="AI18" s="63"/>
       <c r="AJ18" s="36">
         <f t="shared" si="0"/>
-        <v>30.2</v>
+        <v>27.4</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -10988,11 +11023,11 @@
       </c>
       <c r="AO18" s="23">
         <f t="shared" ref="AO18:AO33" si="5">IF(COUNTIF(E18:AI18,"&gt;0")&gt;=15,AVERAGE(E18:AI18),"")</f>
-        <v>27.643478260869575</v>
+        <v>27.63333333333334</v>
       </c>
       <c r="AP18" s="23">
         <f t="shared" si="4"/>
-        <v>1.9949712302657652</v>
+        <v>1.9848263027295303</v>
       </c>
       <c r="AQ18" s="20"/>
     </row>
@@ -11078,7 +11113,9 @@
       <c r="AA19" s="63">
         <v>37.700000000000003</v>
       </c>
-      <c r="AB19" s="63"/>
+      <c r="AB19" s="63">
+        <v>33.4</v>
+      </c>
       <c r="AC19" s="63"/>
       <c r="AD19" s="63"/>
       <c r="AE19" s="63"/>
@@ -11088,7 +11125,7 @@
       <c r="AI19" s="63"/>
       <c r="AJ19" s="36">
         <f t="shared" si="0"/>
-        <v>37.700000000000003</v>
+        <v>33.4</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -11106,11 +11143,11 @@
       </c>
       <c r="AO19" s="23">
         <f t="shared" si="5"/>
-        <v>35.443478260869561</v>
+        <v>35.358333333333327</v>
       </c>
       <c r="AP19" s="23">
         <f t="shared" si="4"/>
-        <v>2.4284624075472578</v>
+        <v>2.3433174800110237</v>
       </c>
       <c r="AQ19" s="20"/>
     </row>
@@ -11196,7 +11233,9 @@
       <c r="AA20" s="63">
         <v>30.8</v>
       </c>
-      <c r="AB20" s="63"/>
+      <c r="AB20" s="63">
+        <v>28.1</v>
+      </c>
       <c r="AC20" s="63"/>
       <c r="AD20" s="63"/>
       <c r="AE20" s="63"/>
@@ -11206,7 +11245,7 @@
       <c r="AI20" s="63"/>
       <c r="AJ20" s="36">
         <f t="shared" si="0"/>
-        <v>30.8</v>
+        <v>28.1</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -11224,11 +11263,11 @@
       </c>
       <c r="AO20" s="23">
         <f t="shared" si="5"/>
-        <v>28.391304347826086</v>
+        <v>28.379166666666666</v>
       </c>
       <c r="AP20" s="23">
         <f t="shared" si="4"/>
-        <v>1.0990687859629666</v>
+        <v>1.086931104803547</v>
       </c>
       <c r="AQ20" s="20"/>
     </row>
@@ -11314,7 +11353,9 @@
       <c r="AA21" s="63">
         <v>24.6</v>
       </c>
-      <c r="AB21" s="63"/>
+      <c r="AB21" s="63">
+        <v>23.4</v>
+      </c>
       <c r="AC21" s="63"/>
       <c r="AD21" s="63"/>
       <c r="AE21" s="63"/>
@@ -11324,7 +11365,7 @@
       <c r="AI21" s="63"/>
       <c r="AJ21" s="36">
         <f t="shared" si="0"/>
-        <v>24.6</v>
+        <v>23.4</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -11342,11 +11383,11 @@
       </c>
       <c r="AO21" s="23">
         <f t="shared" si="5"/>
-        <v>23.160869565217393</v>
+        <v>23.170833333333334</v>
       </c>
       <c r="AP21" s="23">
         <f t="shared" si="4"/>
-        <v>1.2176437587657816</v>
+        <v>1.227607526881723</v>
       </c>
       <c r="AQ21" s="20"/>
     </row>
@@ -11498,7 +11539,9 @@
       <c r="AA23" s="63">
         <v>30.6</v>
       </c>
-      <c r="AB23" s="63"/>
+      <c r="AB23" s="63">
+        <v>29.4</v>
+      </c>
       <c r="AC23" s="63"/>
       <c r="AD23" s="63"/>
       <c r="AE23" s="63"/>
@@ -11508,7 +11551,7 @@
       <c r="AI23" s="63"/>
       <c r="AJ23" s="36">
         <f t="shared" si="0"/>
-        <v>30.6</v>
+        <v>29.4</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -11526,11 +11569,11 @@
       </c>
       <c r="AO23" s="23">
         <f t="shared" si="5"/>
-        <v>27.7</v>
+        <v>27.770833333333332</v>
       </c>
       <c r="AP23" s="23">
         <f t="shared" si="4"/>
-        <v>1.5125310173697279</v>
+        <v>1.5833643507030608</v>
       </c>
       <c r="AQ23" s="20"/>
     </row>
@@ -11616,7 +11659,9 @@
       <c r="AA24" s="63">
         <v>30.1</v>
       </c>
-      <c r="AB24" s="63"/>
+      <c r="AB24" s="63">
+        <v>28.9</v>
+      </c>
       <c r="AC24" s="63"/>
       <c r="AD24" s="63"/>
       <c r="AE24" s="63"/>
@@ -11626,7 +11671,7 @@
       <c r="AI24" s="63"/>
       <c r="AJ24" s="36">
         <f t="shared" si="0"/>
-        <v>30.1</v>
+        <v>28.9</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -11644,11 +11689,11 @@
       </c>
       <c r="AO24" s="23">
         <f t="shared" si="5"/>
-        <v>28.2304347826087</v>
+        <v>28.258333333333336</v>
       </c>
       <c r="AP24" s="23">
         <f t="shared" si="4"/>
-        <v>0.86787397871724892</v>
+        <v>0.89577252944188501</v>
       </c>
       <c r="AQ24" s="20"/>
     </row>
@@ -11734,7 +11779,9 @@
       <c r="AA25" s="63">
         <v>33.700000000000003</v>
       </c>
-      <c r="AB25" s="63"/>
+      <c r="AB25" s="63">
+        <v>32</v>
+      </c>
       <c r="AC25" s="63"/>
       <c r="AD25" s="63"/>
       <c r="AE25" s="63"/>
@@ -11744,7 +11791,7 @@
       <c r="AI25" s="63"/>
       <c r="AJ25" s="36">
         <f t="shared" si="0"/>
-        <v>33.700000000000003</v>
+        <v>32</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11762,11 +11809,11 @@
       </c>
       <c r="AO25" s="23">
         <f t="shared" si="5"/>
-        <v>30.091304347826089</v>
+        <v>30.170833333333334</v>
       </c>
       <c r="AP25" s="23">
         <f t="shared" si="4"/>
-        <v>1.2274014790016601</v>
+        <v>1.3069304645089055</v>
       </c>
       <c r="AQ25" s="20"/>
     </row>
@@ -11852,7 +11899,9 @@
       <c r="AA26" s="63">
         <v>22.7</v>
       </c>
-      <c r="AB26" s="63"/>
+      <c r="AB26" s="63">
+        <v>19.8</v>
+      </c>
       <c r="AC26" s="63"/>
       <c r="AD26" s="63"/>
       <c r="AE26" s="63"/>
@@ -11862,7 +11911,7 @@
       <c r="AI26" s="63"/>
       <c r="AJ26" s="36">
         <f t="shared" si="0"/>
-        <v>22.7</v>
+        <v>19.8</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11880,11 +11929,11 @@
       </c>
       <c r="AO26" s="23">
         <f t="shared" si="5"/>
-        <v>21.330434782608698</v>
+        <v>21.266666666666669</v>
       </c>
       <c r="AP26" s="23">
         <f t="shared" si="4"/>
-        <v>1.9098006134984473</v>
+        <v>1.8460324975564184</v>
       </c>
       <c r="AQ26" s="20"/>
     </row>
@@ -11970,7 +12019,9 @@
       <c r="AA27" s="63">
         <v>21.2</v>
       </c>
-      <c r="AB27" s="63"/>
+      <c r="AB27" s="63">
+        <v>19.8</v>
+      </c>
       <c r="AC27" s="63"/>
       <c r="AD27" s="63"/>
       <c r="AE27" s="63"/>
@@ -11980,7 +12031,7 @@
       <c r="AI27" s="63"/>
       <c r="AJ27" s="36">
         <f t="shared" si="0"/>
-        <v>21.2</v>
+        <v>19.8</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
@@ -11998,11 +12049,11 @@
       </c>
       <c r="AO27" s="23">
         <f t="shared" si="5"/>
-        <v>22.130434782608695</v>
+        <v>22.033333333333331</v>
       </c>
       <c r="AP27" s="23">
         <f t="shared" si="4"/>
-        <v>3.4757664401984165</v>
+        <v>3.3786649909230526</v>
       </c>
       <c r="AQ27" s="20"/>
     </row>
@@ -12088,7 +12139,9 @@
       <c r="AA28" s="63">
         <v>32.299999999999997</v>
       </c>
-      <c r="AB28" s="63"/>
+      <c r="AB28" s="83">
+        <v>32.200000000000003</v>
+      </c>
       <c r="AC28" s="63"/>
       <c r="AD28" s="63"/>
       <c r="AE28" s="63"/>
@@ -12098,7 +12151,7 @@
       <c r="AI28" s="63"/>
       <c r="AJ28" s="36">
         <f t="shared" si="0"/>
-        <v>32.299999999999997</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -12116,11 +12169,11 @@
       </c>
       <c r="AO28" s="23">
         <f t="shared" si="5"/>
-        <v>30.534782608695654</v>
+        <v>30.604166666666671</v>
       </c>
       <c r="AP28" s="23">
         <f t="shared" si="4"/>
-        <v>0.91412582891629413</v>
+        <v>0.98350988688731178</v>
       </c>
       <c r="AQ28" s="20"/>
     </row>
@@ -12270,7 +12323,9 @@
       <c r="AA30" s="63">
         <v>38.200000000000003</v>
       </c>
-      <c r="AB30" s="63"/>
+      <c r="AB30" s="63">
+        <v>35.4</v>
+      </c>
       <c r="AC30" s="63"/>
       <c r="AD30" s="63"/>
       <c r="AE30" s="63"/>
@@ -12280,7 +12335,7 @@
       <c r="AI30" s="63"/>
       <c r="AJ30" s="36">
         <f t="shared" si="0"/>
-        <v>38.200000000000003</v>
+        <v>35.4</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -12298,11 +12353,11 @@
       </c>
       <c r="AO30" s="23">
         <f t="shared" si="5"/>
-        <v>35.986956521739131</v>
+        <v>35.962499999999999</v>
       </c>
       <c r="AP30" s="23">
         <f t="shared" si="4"/>
-        <v>2.5886769518466579</v>
+        <v>2.5642204301075253</v>
       </c>
       <c r="AQ30" s="20"/>
     </row>
@@ -12388,7 +12443,9 @@
       <c r="AA31" s="63">
         <v>25.8</v>
       </c>
-      <c r="AB31" s="63"/>
+      <c r="AB31" s="63">
+        <v>27</v>
+      </c>
       <c r="AC31" s="63"/>
       <c r="AD31" s="63"/>
       <c r="AE31" s="63"/>
@@ -12398,7 +12455,7 @@
       <c r="AI31" s="63"/>
       <c r="AJ31" s="36">
         <f t="shared" si="0"/>
-        <v>25.8</v>
+        <v>27</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -12416,11 +12473,11 @@
       </c>
       <c r="AO31" s="23">
         <f t="shared" si="5"/>
-        <v>25.904347826086951</v>
+        <v>25.949999999999992</v>
       </c>
       <c r="AP31" s="23">
         <f t="shared" si="4"/>
-        <v>1.5843547473575015</v>
+        <v>1.6300069212705424</v>
       </c>
       <c r="AQ31" s="20"/>
     </row>
@@ -12506,7 +12563,9 @@
       <c r="AA32" s="63">
         <v>18.600000000000001</v>
       </c>
-      <c r="AB32" s="63"/>
+      <c r="AB32" s="63">
+        <v>21.4</v>
+      </c>
       <c r="AC32" s="63"/>
       <c r="AD32" s="63"/>
       <c r="AE32" s="63"/>
@@ -12516,7 +12575,7 @@
       <c r="AI32" s="63"/>
       <c r="AJ32" s="36">
         <f t="shared" si="0"/>
-        <v>18.600000000000001</v>
+        <v>21.4</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -12534,11 +12593,11 @@
       </c>
       <c r="AO32" s="23">
         <f t="shared" si="5"/>
-        <v>20.07826086956522</v>
+        <v>20.133333333333336</v>
       </c>
       <c r="AP32" s="23">
         <f t="shared" si="4"/>
-        <v>2.1575867542025584</v>
+        <v>2.2126592179706748</v>
       </c>
       <c r="AQ32" s="20"/>
     </row>
@@ -12624,7 +12683,9 @@
       <c r="AA33" s="63">
         <v>18.8</v>
       </c>
-      <c r="AB33" s="63"/>
+      <c r="AB33" s="63">
+        <v>19.399999999999999</v>
+      </c>
       <c r="AC33" s="63"/>
       <c r="AD33" s="63"/>
       <c r="AE33" s="63"/>
@@ -12634,7 +12695,7 @@
       <c r="AI33" s="63"/>
       <c r="AJ33" s="36">
         <f t="shared" si="0"/>
-        <v>18.8</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -12652,11 +12713,11 @@
       </c>
       <c r="AO33" s="23">
         <f t="shared" si="5"/>
-        <v>18.330434782608695</v>
+        <v>18.374999999999996</v>
       </c>
       <c r="AP33" s="23">
         <f t="shared" si="4"/>
-        <v>1.4348573210613758</v>
+        <v>1.4794225384526776</v>
       </c>
       <c r="AQ33" s="20"/>
       <c r="AT33" s="15"/>
@@ -12794,7 +12855,9 @@
       <c r="AA35" s="63">
         <v>31.6</v>
       </c>
-      <c r="AB35" s="63"/>
+      <c r="AB35" s="63">
+        <v>31.2</v>
+      </c>
       <c r="AC35" s="63"/>
       <c r="AD35" s="63"/>
       <c r="AE35" s="63"/>
@@ -12804,7 +12867,7 @@
       <c r="AI35" s="63"/>
       <c r="AJ35" s="36">
         <f t="shared" si="0"/>
-        <v>31.6</v>
+        <v>31.2</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -12822,11 +12885,11 @@
       </c>
       <c r="AO35" s="23">
         <f>IF(COUNTIF(E35:AI35,"&gt;0")&gt;=15,AVERAGE(E35:AI35),"")</f>
-        <v>31.095652173913049</v>
+        <v>31.100000000000009</v>
       </c>
       <c r="AP35" s="23">
         <f t="shared" si="4"/>
-        <v>0.54128397425314745</v>
+        <v>0.54563180034010728</v>
       </c>
       <c r="AQ35" s="20"/>
       <c r="AT35" s="15"/>
@@ -13031,7 +13094,9 @@
       <c r="AA38" s="63">
         <v>33.9</v>
       </c>
-      <c r="AB38" s="63"/>
+      <c r="AB38" s="63">
+        <v>30.6</v>
+      </c>
       <c r="AC38" s="63"/>
       <c r="AD38" s="63"/>
       <c r="AE38" s="63"/>
@@ -13041,7 +13106,7 @@
       <c r="AI38" s="63"/>
       <c r="AJ38" s="36">
         <f t="shared" si="0"/>
-        <v>33.9</v>
+        <v>30.6</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -13059,11 +13124,11 @@
       </c>
       <c r="AO38" s="23">
         <f>IF(COUNTIF(E38:AI38,"&gt;0")&gt;=15,AVERAGE(E38:AI38),"")</f>
-        <v>33.443478260869561</v>
+        <v>33.324999999999996</v>
       </c>
       <c r="AP38" s="23">
         <f t="shared" si="4"/>
-        <v>1.5064917944253722</v>
+        <v>1.3880135335558066</v>
       </c>
       <c r="AQ38" s="20"/>
       <c r="AT38" s="15"/>
@@ -13150,7 +13215,9 @@
       <c r="AA39" s="63">
         <v>35.6</v>
       </c>
-      <c r="AB39" s="63"/>
+      <c r="AB39" s="63">
+        <v>33.4</v>
+      </c>
       <c r="AC39" s="63"/>
       <c r="AD39" s="63"/>
       <c r="AE39" s="63"/>
@@ -13160,7 +13227,7 @@
       <c r="AI39" s="63"/>
       <c r="AJ39" s="36">
         <f t="shared" si="0"/>
-        <v>35.6</v>
+        <v>33.4</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -13178,11 +13245,11 @@
       </c>
       <c r="AO39" s="23">
         <f t="shared" ref="AO39:AO48" si="7">IF(COUNTIF(E39:AI39,"&gt;0")&gt;=15,AVERAGE(E39:AI39),"")</f>
-        <v>34.221739130434777</v>
+        <v>34.187499999999993</v>
       </c>
       <c r="AP39" s="23">
         <f t="shared" si="4"/>
-        <v>0.79901153186848006</v>
+        <v>0.76477240143369585</v>
       </c>
       <c r="AQ39" s="20"/>
       <c r="AT39" s="15"/>
@@ -13269,7 +13336,9 @@
       <c r="AA40" s="63">
         <v>33.1</v>
       </c>
-      <c r="AB40" s="63"/>
+      <c r="AB40" s="63">
+        <v>29.7</v>
+      </c>
       <c r="AC40" s="63"/>
       <c r="AD40" s="63"/>
       <c r="AE40" s="63"/>
@@ -13279,7 +13348,7 @@
       <c r="AI40" s="63"/>
       <c r="AJ40" s="36">
         <f t="shared" si="0"/>
-        <v>33.1</v>
+        <v>29.7</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -13297,11 +13366,11 @@
       </c>
       <c r="AO40" s="23">
         <f t="shared" si="7"/>
-        <v>31.208695652173912</v>
+        <v>31.145833333333332</v>
       </c>
       <c r="AP40" s="23">
         <f t="shared" si="4"/>
-        <v>0.33031930808789056</v>
+        <v>0.26745698924731087</v>
       </c>
       <c r="AQ40" s="20"/>
       <c r="AT40" s="15"/>
@@ -13382,7 +13451,9 @@
       <c r="AA41" s="63">
         <v>32.799999999999997</v>
       </c>
-      <c r="AB41" s="63"/>
+      <c r="AB41" s="63">
+        <v>32.799999999999997</v>
+      </c>
       <c r="AC41" s="63"/>
       <c r="AD41" s="63"/>
       <c r="AE41" s="63"/>
@@ -13410,11 +13481,11 @@
       </c>
       <c r="AO41" s="23">
         <f t="shared" si="7"/>
-        <v>32.239999999999995</v>
+        <v>32.266666666666666</v>
       </c>
       <c r="AP41" s="23">
         <f t="shared" si="4"/>
-        <v>1.2318094178717054</v>
+        <v>1.2584760845383762</v>
       </c>
       <c r="AQ41" s="20"/>
       <c r="AT41" s="15"/>
@@ -13567,7 +13638,9 @@
       <c r="AA43" s="63">
         <v>33.6</v>
       </c>
-      <c r="AB43" s="63"/>
+      <c r="AB43" s="63">
+        <v>33.4</v>
+      </c>
       <c r="AC43" s="63"/>
       <c r="AD43" s="63"/>
       <c r="AE43" s="63"/>
@@ -13577,7 +13650,7 @@
       <c r="AI43" s="63"/>
       <c r="AJ43" s="36">
         <f t="shared" si="0"/>
-        <v>33.6</v>
+        <v>33.4</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
@@ -13595,11 +13668,11 @@
       </c>
       <c r="AO43" s="23">
         <f t="shared" si="7"/>
-        <v>32.972727272727269</v>
+        <v>32.991304347826087</v>
       </c>
       <c r="AP43" s="23">
         <f t="shared" si="4"/>
-        <v>0.71573460177432224</v>
+        <v>0.73431167687314058</v>
       </c>
       <c r="AQ43" s="20"/>
       <c r="AT43" s="15"/>
@@ -13686,7 +13759,9 @@
       <c r="AA44" s="29">
         <v>31.4</v>
       </c>
-      <c r="AB44" s="29"/>
+      <c r="AB44" s="29">
+        <v>33.200000000000003</v>
+      </c>
       <c r="AC44" s="29"/>
       <c r="AD44" s="29"/>
       <c r="AE44" s="63"/>
@@ -13696,7 +13771,7 @@
       <c r="AI44" s="63"/>
       <c r="AJ44" s="36">
         <f t="shared" si="0"/>
-        <v>31.4</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="1"/>
@@ -13714,11 +13789,11 @@
       </c>
       <c r="AO44" s="23">
         <f t="shared" si="7"/>
-        <v>31.817391304347829</v>
+        <v>31.875000000000004</v>
       </c>
       <c r="AP44" s="23">
         <f t="shared" si="4"/>
-        <v>0.73070430350620796</v>
+        <v>0.78831299915838215</v>
       </c>
       <c r="AQ44" s="20"/>
       <c r="AT44" s="15"/>
@@ -13805,7 +13880,9 @@
       <c r="AA45" s="63">
         <v>33.4</v>
       </c>
-      <c r="AB45" s="63"/>
+      <c r="AB45" s="63">
+        <v>32.4</v>
+      </c>
       <c r="AC45" s="63"/>
       <c r="AD45" s="63"/>
       <c r="AE45" s="63"/>
@@ -13815,7 +13892,7 @@
       <c r="AI45" s="63"/>
       <c r="AJ45" s="36">
         <f t="shared" si="0"/>
-        <v>33.4</v>
+        <v>32.4</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -13833,11 +13910,11 @@
       </c>
       <c r="AO45" s="23">
         <f t="shared" si="7"/>
-        <v>32.947826086956525</v>
+        <v>32.925000000000004</v>
       </c>
       <c r="AP45" s="23">
         <f t="shared" si="4"/>
-        <v>1.3526313163609345</v>
+        <v>1.329805229404414</v>
       </c>
       <c r="AQ45" s="20"/>
       <c r="AT45" s="15"/>
@@ -14056,7 +14133,9 @@
       <c r="AA48" s="63">
         <v>31.4</v>
       </c>
-      <c r="AB48" s="63"/>
+      <c r="AB48" s="63">
+        <v>34.299999999999997</v>
+      </c>
       <c r="AC48" s="63"/>
       <c r="AD48" s="63"/>
       <c r="AE48" s="63"/>
@@ -14066,7 +14145,7 @@
       <c r="AI48" s="63"/>
       <c r="AJ48" s="36">
         <f t="shared" si="0"/>
-        <v>31.4</v>
+        <v>34.299999999999997</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -14084,11 +14163,11 @@
       </c>
       <c r="AO48" s="23">
         <f t="shared" si="7"/>
-        <v>32.830434782608698</v>
+        <v>32.891666666666673</v>
       </c>
       <c r="AP48" s="23">
         <f t="shared" si="4"/>
-        <v>0.83824553529686696</v>
+        <v>0.8994774193548416</v>
       </c>
       <c r="AQ48" s="20"/>
     </row>
@@ -16221,7 +16300,7 @@
       <formula>100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O17:O28 T17:W28 Y17:Y28 AC17:AC28 AF17:AF28 E17:G33 Z17:AB33 AH17:AI33 AD23:AD28 O25:Q25 S25:Y25 AC25:AG25 E35:G36 I35:K36 M35:M36 O35:AC36 AE35:AI36 M38:M42 O38:AC42 AE38:AI42 E38:G46 I38:K46 E5:G15 I5:K15 M5:M15 I17:K33 M17:M33 R17:R33 O29:Q33 S29:Y33 AC29:AG33 M43:AI43 M44:Q44 AC44 S44:AB45 AE44:AI45 R44:R46 M45:M46 E48:G48 I48:K48 M48 AC38:AG41 AC5:AG13 AD5:AI15 AE17:AG22 AG17:AG24 AG26:AG28 AC27:AG27 AC35:AG35 AC45:AG45 O48:AI48 S17:Y22 S17:T24 O5:AB15 P26:Q28 S26:T28 O45:Q46 S46:AI46 AE17:AE24 AE26:AE28 X17:X24 X26:X28 X27:Y27 O17:Q22 P17:Q24 AD17:AD21 AC6:AC15 AJ16:AK16 AJ34:AM34 AJ37:AM37">
+  <conditionalFormatting sqref="O17:O28 T17:W28 Y17:Y28 AC17:AC28 AF17:AF28 E17:G33 AH17:AI33 AD23:AD28 O25:Q25 S25:Y25 AC25:AG25 E35:G36 I35:K36 M35:M36 O35:AC36 AE35:AI36 M38:M42 O38:AC42 AE38:AI42 E38:G46 I38:K46 E5:G15 I5:K15 M5:M15 I17:K33 M17:M33 R17:R33 O29:Q33 S29:Y33 AC29:AG33 M43:AI43 M44:Q44 AC44 S44:AB45 AE44:AI45 R44:R46 M45:M46 E48:G48 I48:K48 M48 AC38:AG41 AC5:AG13 AD5:AI15 AE17:AG22 AG17:AG24 AG26:AG28 AC27:AG27 AC35:AG35 AC45:AG45 O48:AI48 S17:Y22 S17:T24 O5:AB15 P26:Q28 S26:T28 O45:Q46 S46:AI46 AE17:AE24 AE26:AE28 X17:X24 X26:X28 X27:Y27 O17:Q22 P17:Q24 AD17:AD21 AC6:AC15 AJ16:AK16 AJ34:AM34 AJ37:AM37 Z17:AB33">
     <cfRule type="cellIs" dxfId="413" priority="3481" stopIfTrue="1" operator="between">
       <formula>45</formula>
       <formula>100</formula>
@@ -16946,7 +17025,7 @@
       <formula>NOT(ISERROR(SEARCH("sd",X22)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X5:Y15 AA5:AB15 Y17:Y28 AA17:AB28 X27:Z27 AC27:AI27 X30:Y33 AA30:AB33 X35:Y36 AA35:AB36 X38:Y42 AA38:AB42 X45:Y45 AA45:AB45 X46:AI46 X48:Y48 AA48:AB48">
+  <conditionalFormatting sqref="X5:Y15 AA5:AB15 Y17:Y28 AA17:AB28 X27:Z27 AC27:AI27 X30:Y33 X35:Y36 AA35:AB36 X38:Y42 AA38:AB42 X45:Y45 AA45:AB45 X46:AI46 X48:Y48 AA48:AB48 AA30:AB33">
     <cfRule type="cellIs" dxfId="230" priority="1644" stopIfTrue="1" operator="between">
       <formula>-9.9</formula>
       <formula>-10</formula>
@@ -16995,7 +17074,7 @@
       <formula>NOT(ISERROR(SEARCH("sd",X42)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y17:Y28 AA17:AB28 X35:Y36 AA35:AB36 X38:Y42 AA38:AB42 AC27:AI27 X5:Y15 AA5:AB15 X27:Z27 X30:Y33 AA30:AB33 X45:Y45 AA45:AB45 X46:AI46 X48:Y48 AA48:AB48">
+  <conditionalFormatting sqref="Y17:Y28 AA17:AB28 X35:Y36 AA35:AB36 X38:Y42 AA38:AB42 AC27:AI27 X5:Y15 AA5:AB15 X27:Z27 X30:Y33 X45:Y45 AA45:AB45 X46:AI46 X48:Y48 AA48:AB48 AA30:AB33">
     <cfRule type="cellIs" dxfId="218" priority="1640" stopIfTrue="1" operator="between">
       <formula>45</formula>
       <formula>100</formula>
@@ -17030,12 +17109,12 @@
       <formula>NOT(ISERROR(SEARCH("sd",Y42)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC5:AG5 E5:G15 I5:K15 M5:M15 O5:AB15 AD5:AI15 AC6:AC15 AC12:AG13 AJ16:AK16 AD17:AD21 P17:Q24 S17:T24 X17:X24 AE17:AE24 AG17:AG24 O17:O28 T17:W28 Y17:Y28 AC17:AC28 AF17:AF28 E17:G33 I17:K33 M17:M33 R17:R33 Z17:AB33 AH17:AI33 O22:Q22 S22:Y22 AE22:AG22 AD23:AD28 O25:Q25 S25:Y25 AC25:AG25 P26:Q28 S26:T28 X26:X28 AE26:AE28 AG26:AG28 X27:Y27 AC27:AG27 O29:Q33 S29:Y33 AC29:AG33 AJ34:AM34 AC35:AG35 E35:G36 I35:K36 M35:M36 O35:AC36 AE35:AI36 AJ37:AM37 AC38:AG41 M38:M42 O38:AC42 AE38:AI42 E38:G46 I38:K46 M43:AI43 M44:Q44 AC44 S44:AB45 AE44:AI45 R44:R46 AC45:AG45 M45:M46 O45:Q46 S46:AI46 E48:G48 I48:K48 M48 O48:AI48">
+  <conditionalFormatting sqref="AC5:AG5 E5:G15 I5:K15 M5:M15 O5:AB15 AD5:AI15 AC6:AC15 AC12:AG13 AJ16:AK16 AD17:AD21 P17:Q24 S17:T24 X17:X24 AE17:AE24 AG17:AG24 O17:O28 T17:W28 Y17:Y28 AC17:AC28 AF17:AF28 E17:G33 I17:K33 M17:M33 R17:R33 AH17:AI33 O22:Q22 S22:Y22 AE22:AG22 AD23:AD28 O25:Q25 S25:Y25 AC25:AG25 P26:Q28 S26:T28 X26:X28 AE26:AE28 AG26:AG28 X27:Y27 AC27:AG27 O29:Q33 S29:Y33 AC29:AG33 AJ34:AM34 AC35:AG35 E35:G36 I35:K36 M35:M36 O35:AC36 AE35:AI36 AJ37:AM37 AC38:AG41 M38:M42 O38:AC42 AE38:AI42 E38:G46 I38:K46 M43:AI43 M44:Q44 AC44 S44:AB45 AE44:AI45 R44:R46 AC45:AG45 M45:M46 O45:Q46 S46:AI46 E48:G48 I48:K48 M48 O48:AI48 Z17:AB33">
     <cfRule type="cellIs" dxfId="210" priority="3526" stopIfTrue="1" operator="equal">
       <formula>"SD"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC5:AG13 E5:G15 I5:K15 M5:M15 O5:AB15 AD5:AI15 AC6:AC15 AJ16:AK16 AD17:AD21 O17:Q22 S17:Y22 AE17:AG22 P17:Q24 S17:T24 X17:X24 AE17:AE24 AG17:AG24 O17:O28 T17:W28 Y17:Y28 AC17:AC28 AF17:AF28 E17:G33 I17:K33 M17:M33 R17:R33 Z17:AB33 AH17:AI33 AD23:AD28 O25:Q25 S25:Y25 AC25:AG25 P26:Q28 S26:T28 X26:X28 AE26:AE28 AG26:AG28 X27:Y27 AC27:AG27 O29:Q33 S29:Y33 AC29:AG33 AJ34:AM34 AC35:AG35 E35:G36 I35:K36 M35:M36 O35:AC36 AE35:AI36 AJ37:AM37 AC38:AG41 M38:M42 O38:AC42 AE38:AI42 E38:G46 I38:K46 M43:AI43 M44:Q44 AC44 S44:AB45 AE44:AI45 R44:R46 AC45:AG45 M45:M46 O45:Q46 S46:AI46 E48:G48 I48:K48 M48 O48:AI48">
+  <conditionalFormatting sqref="AC5:AG13 E5:G15 I5:K15 M5:M15 O5:AB15 AD5:AI15 AC6:AC15 AJ16:AK16 AD17:AD21 O17:Q22 S17:Y22 AE17:AG22 P17:Q24 S17:T24 X17:X24 AE17:AE24 AG17:AG24 O17:O28 T17:W28 Y17:Y28 AC17:AC28 AF17:AF28 E17:G33 I17:K33 M17:M33 R17:R33 AH17:AI33 AD23:AD28 O25:Q25 S25:Y25 AC25:AG25 P26:Q28 S26:T28 X26:X28 AE26:AE28 AG26:AG28 X27:Y27 AC27:AG27 O29:Q33 S29:Y33 AC29:AG33 AJ34:AM34 AC35:AG35 E35:G36 I35:K36 M35:M36 O35:AC36 AE35:AI36 AJ37:AM37 AC38:AG41 M38:M42 O38:AC42 AE38:AI42 E38:G46 I38:K46 M43:AI43 M44:Q44 AC44 S44:AB45 AE44:AI45 R44:R46 AC45:AG45 M45:M46 O45:Q46 S46:AI46 E48:G48 I48:K48 M48 O48:AI48 Z17:AB33">
     <cfRule type="cellIs" dxfId="209" priority="3482" stopIfTrue="1" operator="equal">
       <formula>"40.0"</formula>
     </cfRule>

</xml_diff>